<commit_message>
improving species C stock estimates
</commit_message>
<xml_diff>
--- a/Carbon_Calculations/IPCC_Carbon_Calculations.xlsx
+++ b/Carbon_Calculations/IPCC_Carbon_Calculations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uillinoisedu-my.sharepoint.com/personal/cmptrsn2_illinois_edu/Documents/Chapter2/Floodplain-Experiment-Repo/Tree_Analysis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uillinoisedu-my.sharepoint.com/personal/cmptrsn2_illinois_edu/Documents/Ch2_Floodplain_Experiment/Floodplain-Experiment-Repo/Carbon_Calculations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1385" documentId="8_{81C5A17B-0AA7-4E1F-9EEB-1F73114DAE67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B132E2AB-BAAE-4655-8D4E-2FDF1964FB49}"/>
+  <xr:revisionPtr revIDLastSave="1386" documentId="8_{81C5A17B-0AA7-4E1F-9EEB-1F73114DAE67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9AFEF6A6-EBC4-458C-B563-8E003EF77F47}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-3420" windowWidth="29040" windowHeight="15990" xr2:uid="{2C906CBC-631A-4B26-833B-3AA2F3C7757D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{2C906CBC-631A-4B26-833B-3AA2F3C7757D}"/>
   </bookViews>
   <sheets>
     <sheet name="Henry County estimates" sheetId="1" r:id="rId1"/>
@@ -210,9 +210,6 @@
     <t>Dead wood C concentration (%)</t>
   </si>
   <si>
-    <t>Harmon et al. (2013): Assumed angiosperms, do not know decay class or if standing v. downed</t>
-  </si>
-  <si>
     <t>Decay class</t>
   </si>
   <si>
@@ -262,6 +259,9 @@
   </si>
   <si>
     <t>Total live woody carbon</t>
+  </si>
+  <si>
+    <t>Harmon et al. (2013): Assumed angiosperms, decay class 3, do not know if standing v. downed</t>
   </si>
 </sst>
 </file>
@@ -338,6 +338,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -658,19 +662,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ECBA9F9-5B1E-4DE3-BE7E-98B24B386112}">
   <dimension ref="A1:H42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.85546875" customWidth="1"/>
-    <col min="2" max="2" width="29.7109375" customWidth="1"/>
+    <col min="1" max="1" width="22.88671875" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" customWidth="1"/>
     <col min="3" max="3" width="59" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" customWidth="1"/>
-    <col min="5" max="6" width="15.28515625" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" customWidth="1"/>
-    <col min="8" max="8" width="48.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" customWidth="1"/>
+    <col min="5" max="6" width="15.33203125" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" customWidth="1"/>
+    <col min="8" max="8" width="48.88671875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
@@ -696,7 +700,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
@@ -721,10 +725,10 @@
         <v>0.12</v>
       </c>
       <c r="H2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
@@ -750,7 +754,7 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>8</v>
       </c>
@@ -764,7 +768,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>27</v>
       </c>
@@ -783,12 +787,12 @@
         <v>0.17</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C6" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C7" t="s">
         <v>37</v>
       </c>
@@ -808,7 +812,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C8" t="s">
         <v>30</v>
       </c>
@@ -819,7 +823,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C9" t="s">
         <v>56</v>
       </c>
@@ -833,10 +837,10 @@
         <v>0.52</v>
       </c>
       <c r="H9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C10" t="s">
         <v>39</v>
       </c>
@@ -847,7 +851,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C11" t="s">
         <v>40</v>
       </c>
@@ -864,7 +868,7 @@
         <v>0.36088000000000003</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C12" t="s">
         <v>31</v>
       </c>
@@ -881,7 +885,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C13" t="s">
         <v>32</v>
       </c>
@@ -895,7 +899,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C14" t="s">
         <v>23</v>
       </c>
@@ -912,7 +916,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C15" t="s">
         <v>33</v>
       </c>
@@ -929,7 +933,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C16" t="s">
         <v>48</v>
       </c>
@@ -943,7 +947,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C17" t="s">
         <v>53</v>
       </c>
@@ -960,7 +964,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C18" t="s">
         <v>46</v>
       </c>
@@ -974,7 +978,7 @@
         <v>0.37</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C19" t="s">
         <v>54</v>
       </c>
@@ -988,7 +992,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>1</v>
       </c>
@@ -1008,7 +1012,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>2</v>
       </c>
@@ -1028,7 +1032,7 @@
         <v>75.55680000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B23" s="5" t="s">
         <v>28</v>
       </c>
@@ -1045,7 +1049,7 @@
         <v>87.12</v>
       </c>
     </row>
-    <row r="24" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B24" s="5" t="s">
         <v>0</v>
       </c>
@@ -1059,10 +1063,10 @@
         <v>88</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>21</v>
       </c>
@@ -1082,7 +1086,7 @@
         <v>15.5</v>
       </c>
     </row>
-    <row r="26" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B26" s="5" t="s">
         <v>17</v>
       </c>
@@ -1099,7 +1103,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="27" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>16</v>
       </c>
@@ -1119,7 +1123,7 @@
         <v>9.0220000000000002</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B28" s="5" t="s">
         <v>20</v>
       </c>
@@ -1136,9 +1140,9 @@
         <v>18.044</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B29" t="s">
         <v>19</v>
@@ -1156,7 +1160,7 @@
         <v>24.521999999999998</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>20</v>
       </c>
@@ -1173,7 +1177,7 @@
         <v>49.043999999999997</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>42</v>
       </c>
@@ -1193,7 +1197,7 @@
         <v>197.5</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>22</v>
       </c>
@@ -1210,7 +1214,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="33" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>43</v>
       </c>
@@ -1230,7 +1234,7 @@
         <v>98.75</v>
       </c>
     </row>
-    <row r="34" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B34" s="5" t="s">
         <v>22</v>
       </c>
@@ -1247,7 +1251,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>47</v>
       </c>
@@ -1267,7 +1271,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>22</v>
       </c>
@@ -1284,7 +1288,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="37" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>44</v>
       </c>
@@ -1304,7 +1308,7 @@
         <v>43.45</v>
       </c>
     </row>
-    <row r="38" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B38" s="5" t="s">
         <v>22</v>
       </c>
@@ -1321,9 +1325,9 @@
         <v>44</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B39" t="s">
         <v>18</v>
@@ -1341,7 +1345,7 @@
         <v>142.19999999999999</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>22</v>
       </c>
@@ -1358,7 +1362,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="41" spans="1:5" s="5" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" s="5" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>41</v>
       </c>
@@ -1378,7 +1382,7 @@
         <v>253.84199999999998</v>
       </c>
     </row>
-    <row r="42" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B42" s="5" t="s">
         <v>26</v>
       </c>
@@ -1403,55 +1407,55 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C7E7DBA-8DFD-4420-810D-ADC70A6F6B52}">
   <dimension ref="A1:K13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1" t="s">
         <v>62</v>
       </c>
-      <c r="G1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" t="s">
         <v>58</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>59</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>60</v>
       </c>
-      <c r="D2" t="s">
-        <v>61</v>
-      </c>
       <c r="E2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F2" t="s">
         <v>67</v>
       </c>
-      <c r="F2" t="s">
-        <v>68</v>
-      </c>
       <c r="G2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H2" t="s">
         <v>59</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>60</v>
       </c>
-      <c r="I2" t="s">
-        <v>61</v>
-      </c>
       <c r="J2" t="s">
+        <v>66</v>
+      </c>
+      <c r="K2" t="s">
         <v>67</v>
       </c>
-      <c r="K2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>0</v>
       </c>
@@ -1472,7 +1476,7 @@
         <v>48.6</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
@@ -1509,7 +1513,7 @@
         <v>48.6</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2</v>
       </c>
@@ -1546,7 +1550,7 @@
         <v>48.6</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>3</v>
       </c>
@@ -1583,7 +1587,7 @@
         <v>49.2</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>4</v>
       </c>
@@ -1620,7 +1624,7 @@
         <v>49.4</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>5</v>
       </c>
@@ -1641,9 +1645,9 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C9">
         <f>SUM(C3:C8)</f>
@@ -1662,9 +1666,9 @@
         <v>531.4</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C10">
         <f>C9+H9</f>
@@ -1675,27 +1679,27 @@
         <v>5639.5</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D11" s="4">
         <f>D10/C10/100</f>
         <v>0.47792372881355932</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D12">
         <f>MIN(E3:E8,J4:J7)/100</f>
         <v>0.434</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D13">
         <f>MAX(F3:F8,K4:K7)/100</f>

</xml_diff>